<commit_message>
Add figure 13 that shows average weekday and weekend on- and  off-peak prices  for  months of March - May and October
</commit_message>
<xml_diff>
--- a/Energy Rates_2014.xlsx
+++ b/Energy Rates_2014.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B87275D-0C4B-4B77-B82F-358FCE105510}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72BBD742-AC03-411F-85F2-01D25BB80BFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-57720" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="-1260" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="12" r:id="rId1"/>
@@ -236,9 +236,6 @@
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -247,6 +244,9 @@
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -10894,30 +10894,30 @@
       <c r="A4" t="s">
         <v>24</v>
       </c>
-      <c r="C4" s="17">
+      <c r="C4" s="16">
         <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="15" t="s">
+      <c r="A5" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="C5" s="16" t="s">
+      <c r="C5" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="16" t="s">
+      <c r="D5" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="E5" s="16" t="s">
+      <c r="E5" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="G5" s="16" t="s">
+      <c r="G5" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="H5" s="16" t="s">
+      <c r="H5" s="15" t="s">
         <v>25</v>
       </c>
     </row>
@@ -10925,28 +10925,28 @@
       <c r="A6" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="17">
+      <c r="B6" s="16">
         <f>AVERAGE(March!H5:H12)</f>
         <v>34.699513831553666</v>
       </c>
-      <c r="C6" s="18">
+      <c r="C6" s="17">
         <f>MIN(March!$H$13:$H$28)</f>
         <v>49.437253253625322</v>
       </c>
-      <c r="D6" s="18">
+      <c r="D6" s="17">
         <f>MAX(March!$H$13:$H$28)</f>
         <v>72.901798874118612</v>
       </c>
-      <c r="E6" s="18">
+      <c r="E6" s="17">
         <f>AVERAGE(March!$H$13:$H$28)</f>
         <v>58.52242346956902</v>
       </c>
-      <c r="G6" s="18">
+      <c r="G6" s="17">
         <f>B6+$C$4</f>
         <v>64.699513831553674</v>
       </c>
-      <c r="H6" s="18">
-        <f>E6+$C$4</f>
+      <c r="H6" s="17">
+        <f t="shared" ref="H6:H13" si="0">E6+$C$4</f>
         <v>88.52242346956902</v>
       </c>
     </row>
@@ -10954,28 +10954,28 @@
       <c r="A7" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="17">
+      <c r="B7" s="16">
         <f>AVERAGE(April!H5:H13)</f>
         <v>30.742340534310568</v>
       </c>
-      <c r="C7" s="18">
+      <c r="C7" s="17">
         <f>MIN(April!$H$13:$H$28)</f>
         <v>41.434816092364287</v>
       </c>
-      <c r="D7" s="18">
+      <c r="D7" s="17">
         <f>MAX(April!$H$13:$H$28)</f>
         <v>65.112841412882219</v>
       </c>
-      <c r="E7" s="18">
+      <c r="E7" s="17">
         <f>AVERAGE(April!$H$13:$H$28)</f>
         <v>55.050518027815997</v>
       </c>
-      <c r="G7" s="18">
-        <f t="shared" ref="G7:G13" si="0">B7+$C$4</f>
+      <c r="G7" s="17">
+        <f t="shared" ref="G7:G13" si="1">B7+$C$4</f>
         <v>60.742340534310571</v>
       </c>
-      <c r="H7" s="18">
-        <f>E7+$C$4</f>
+      <c r="H7" s="17">
+        <f t="shared" si="0"/>
         <v>85.050518027815997</v>
       </c>
     </row>
@@ -10983,28 +10983,28 @@
       <c r="A8" t="s">
         <v>3</v>
       </c>
-      <c r="B8" s="17">
+      <c r="B8" s="16">
         <f>AVERAGE(May!H5:H12)</f>
         <v>26.497999818602068</v>
       </c>
-      <c r="C8" s="18">
+      <c r="C8" s="17">
         <f>MIN(May!$H$13:$H$28)</f>
         <v>39.150558992560093</v>
       </c>
-      <c r="D8" s="18">
+      <c r="D8" s="17">
         <f>MAX(May!$H$13:$H$28)</f>
         <v>68.331203254274541</v>
       </c>
-      <c r="E8" s="18">
+      <c r="E8" s="17">
         <f>AVERAGE(May!$H$13:$H$28)</f>
         <v>56.571035064133454</v>
       </c>
-      <c r="G8" s="18">
+      <c r="G8" s="17">
+        <f t="shared" si="1"/>
+        <v>56.497999818602068</v>
+      </c>
+      <c r="H8" s="17">
         <f t="shared" si="0"/>
-        <v>56.497999818602068</v>
-      </c>
-      <c r="H8" s="18">
-        <f>E8+$C$4</f>
         <v>86.571035064133454</v>
       </c>
     </row>
@@ -11012,28 +11012,28 @@
       <c r="A9" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="17">
+      <c r="B9" s="16">
         <f>AVERAGE(June!H$5:H$12)</f>
         <v>27.246566631171877</v>
       </c>
-      <c r="C9" s="18">
+      <c r="C9" s="17">
         <f>MIN(June!$H$14:$H$29)</f>
         <v>55.469334102638705</v>
       </c>
-      <c r="D9" s="18">
+      <c r="D9" s="17">
         <f>MAX(June!$H$14:$H$29)</f>
         <v>69.225430424419073</v>
       </c>
-      <c r="E9" s="18">
+      <c r="E9" s="17">
         <f>AVERAGE(June!$H$14:$H$29)</f>
         <v>62.347382263528885</v>
       </c>
-      <c r="G9" s="18">
+      <c r="G9" s="17">
+        <f t="shared" si="1"/>
+        <v>57.246566631171873</v>
+      </c>
+      <c r="H9" s="17">
         <f t="shared" si="0"/>
-        <v>57.246566631171873</v>
-      </c>
-      <c r="H9" s="18">
-        <f>E9+$C$4</f>
         <v>92.347382263528885</v>
       </c>
     </row>
@@ -11041,28 +11041,28 @@
       <c r="A10" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="17">
+      <c r="B10" s="16">
         <f>AVERAGE(July!H$5:H$12)</f>
         <v>29.783034890110805</v>
       </c>
-      <c r="C10" s="18">
+      <c r="C10" s="17">
         <f>MIN(July!$H$14:$H$29)</f>
         <v>50.455663052098267</v>
       </c>
-      <c r="D10" s="18">
+      <c r="D10" s="17">
         <f>MAX(July!$H$14:$H$29)</f>
         <v>105.7903671905766</v>
       </c>
-      <c r="E10" s="18">
+      <c r="E10" s="17">
         <f>AVERAGE(July!$H$14:$H$29)</f>
         <v>77.939790165392921</v>
       </c>
-      <c r="G10" s="18">
+      <c r="G10" s="17">
+        <f t="shared" si="1"/>
+        <v>59.783034890110805</v>
+      </c>
+      <c r="H10" s="17">
         <f t="shared" si="0"/>
-        <v>59.783034890110805</v>
-      </c>
-      <c r="H10" s="18">
-        <f>E10+$C$4</f>
         <v>107.93979016539292</v>
       </c>
     </row>
@@ -11070,28 +11070,28 @@
       <c r="A11" t="s">
         <v>22</v>
       </c>
-      <c r="B11" s="17">
+      <c r="B11" s="16">
         <f>AVERAGE(August!H$5:H$12)</f>
         <v>37.291815900739664</v>
       </c>
-      <c r="C11" s="18">
+      <c r="C11" s="17">
         <f>MIN(August!$H$13:$H$28)</f>
         <v>56.415215712703464</v>
       </c>
-      <c r="D11" s="18">
+      <c r="D11" s="17">
         <f>MAX(August!$H$13:$H$28)</f>
         <v>98.736673005401059</v>
       </c>
-      <c r="E11" s="18">
+      <c r="E11" s="17">
         <f>AVERAGE(August!$H$13:$H$28)</f>
         <v>77.510850185651449</v>
       </c>
-      <c r="G11" s="18">
+      <c r="G11" s="17">
+        <f t="shared" si="1"/>
+        <v>67.291815900739664</v>
+      </c>
+      <c r="H11" s="17">
         <f t="shared" si="0"/>
-        <v>67.291815900739664</v>
-      </c>
-      <c r="H11" s="18">
-        <f>E11+$C$4</f>
         <v>107.51085018565145</v>
       </c>
     </row>
@@ -11099,28 +11099,28 @@
       <c r="A12" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="17">
+      <c r="B12" s="16">
         <f>AVERAGE(September!H$5:H$12)</f>
         <v>38.661257418652681</v>
       </c>
-      <c r="C12" s="18">
+      <c r="C12" s="17">
         <f>MIN(September!$H$13:$H$28)</f>
         <v>54.043362670844516</v>
       </c>
-      <c r="D12" s="18">
+      <c r="D12" s="17">
         <f>MAX(September!$H$13:$H$28)</f>
         <v>84.369596466058951</v>
       </c>
-      <c r="E12" s="18">
+      <c r="E12" s="17">
         <f>AVERAGE(September!$H$13:$H$28)</f>
         <v>68.941412614337224</v>
       </c>
-      <c r="G12" s="18">
+      <c r="G12" s="17">
+        <f t="shared" si="1"/>
+        <v>68.661257418652681</v>
+      </c>
+      <c r="H12" s="17">
         <f t="shared" si="0"/>
-        <v>68.661257418652681</v>
-      </c>
-      <c r="H12" s="18">
-        <f>E12+$C$4</f>
         <v>98.941412614337224</v>
       </c>
     </row>
@@ -11128,28 +11128,28 @@
       <c r="A13" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="17">
+      <c r="B13" s="16">
         <f>AVERAGE(October!H$5:H$12)</f>
         <v>35.982148506817737</v>
       </c>
-      <c r="C13" s="18">
+      <c r="C13" s="17">
         <f>MIN(October!$H$13:$H$28)</f>
         <v>54.1428800013555</v>
       </c>
-      <c r="D13" s="18">
+      <c r="D13" s="17">
         <f>MAX(October!$H$13:$H$28)</f>
         <v>82.540478984940776</v>
       </c>
-      <c r="E13" s="18">
+      <c r="E13" s="17">
         <f>AVERAGE(October!$H$13:$H$28)</f>
         <v>64.953451257263765</v>
       </c>
-      <c r="G13" s="18">
+      <c r="G13" s="17">
+        <f t="shared" si="1"/>
+        <v>65.982148506817737</v>
+      </c>
+      <c r="H13" s="17">
         <f t="shared" si="0"/>
-        <v>65.982148506817737</v>
-      </c>
-      <c r="H13" s="18">
-        <f>E13+$C$4</f>
         <v>94.953451257263765</v>
       </c>
     </row>
@@ -13697,19 +13697,19 @@
       <c r="E4" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="F4" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="G4" s="14"/>
-      <c r="H4" s="14"/>
+      <c r="G4" s="18"/>
+      <c r="H4" s="18"/>
       <c r="I4" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="J4" s="14" t="s">
+      <c r="J4" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="K4" s="14"/>
-      <c r="L4" s="14"/>
+      <c r="K4" s="18"/>
+      <c r="L4" s="18"/>
       <c r="M4" s="6"/>
     </row>
     <row r="5" spans="2:13" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Fix error in calculating weekly average prices
</commit_message>
<xml_diff>
--- a/Energy Rates_2014.xlsx
+++ b/Energy Rates_2014.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72BBD742-AC03-411F-85F2-01D25BB80BFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15A8B50D-F342-432E-85B9-4CCBC0B3A35E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="57480" yWindow="-1260" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="41">
   <si>
     <t>Price Profiles for Generation Shaping ($/MWh)--Simulation Info Tab, Monday Hourly Values</t>
   </si>
@@ -131,6 +131,39 @@
   <si>
     <t>Summary of Min, Max, and Average on-peak weekday contract Glen Canyon Dam energy prices ($/MW-hour)</t>
   </si>
+  <si>
+    <t>Rind and Rosenberg</t>
+  </si>
+  <si>
+    <t>2024 - Yackulic</t>
+  </si>
+  <si>
+    <t>MonthWord</t>
+  </si>
+  <si>
+    <t>Weekday_OffPeak</t>
+  </si>
+  <si>
+    <t>Weekday_OnPeak</t>
+  </si>
+  <si>
+    <t>Weekend_OffPeak</t>
+  </si>
+  <si>
+    <t>Weekend_OnPeak</t>
+  </si>
+  <si>
+    <t>Off-Peak</t>
+  </si>
+  <si>
+    <t>Rind Rosenberg</t>
+  </si>
+  <si>
+    <t>Yackulic</t>
+  </si>
+  <si>
+    <t>On-peak</t>
+  </si>
 </sst>
 </file>
 
@@ -217,7 +250,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -245,6 +278,9 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -10873,32 +10909,45 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E4AFA8A-3ECC-44AF-AF5D-50FFF5439E6C}">
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:T13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="7" max="7" width="8.81640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="2.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>24</v>
       </c>
       <c r="C4" s="16">
         <v>30</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="G4" t="s">
+        <v>30</v>
+      </c>
+      <c r="J4" t="s">
+        <v>31</v>
+      </c>
+      <c r="P4" t="s">
+        <v>37</v>
+      </c>
+      <c r="S4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
         <v>16</v>
       </c>
@@ -10920,8 +10969,35 @@
       <c r="H5" s="15" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J5" t="s">
+        <v>32</v>
+      </c>
+      <c r="K5" t="s">
+        <v>33</v>
+      </c>
+      <c r="L5" t="s">
+        <v>34</v>
+      </c>
+      <c r="M5" t="s">
+        <v>35</v>
+      </c>
+      <c r="N5" t="s">
+        <v>36</v>
+      </c>
+      <c r="P5" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q5" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="S5" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="T5" s="8" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -10949,8 +11025,40 @@
         <f t="shared" ref="H6:H13" si="0">E6+$C$4</f>
         <v>88.52242346956902</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J6" t="s">
+        <v>12</v>
+      </c>
+      <c r="K6">
+        <v>39.5</v>
+      </c>
+      <c r="L6">
+        <v>53.3</v>
+      </c>
+      <c r="M6">
+        <v>23.4</v>
+      </c>
+      <c r="N6">
+        <v>46.2</v>
+      </c>
+      <c r="P6" s="19">
+        <f>G6</f>
+        <v>64.699513831553674</v>
+      </c>
+      <c r="Q6" s="6">
+        <f>K6</f>
+        <v>39.5</v>
+      </c>
+      <c r="R6" s="6"/>
+      <c r="S6" s="19">
+        <f>H6</f>
+        <v>88.52242346956902</v>
+      </c>
+      <c r="T6" s="6">
+        <f>L6</f>
+        <v>53.3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -10978,8 +11086,40 @@
         <f t="shared" si="0"/>
         <v>85.050518027815997</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J7" t="s">
+        <v>19</v>
+      </c>
+      <c r="K7">
+        <v>33.5</v>
+      </c>
+      <c r="L7">
+        <v>53.9</v>
+      </c>
+      <c r="M7">
+        <v>16.5</v>
+      </c>
+      <c r="N7">
+        <v>46.3</v>
+      </c>
+      <c r="P7" s="19">
+        <f t="shared" ref="P7:P13" si="2">G7</f>
+        <v>60.742340534310571</v>
+      </c>
+      <c r="Q7" s="6">
+        <f t="shared" ref="Q7:Q13" si="3">K7</f>
+        <v>33.5</v>
+      </c>
+      <c r="R7" s="6"/>
+      <c r="S7" s="19">
+        <f t="shared" ref="S7:S13" si="4">H7</f>
+        <v>85.050518027815997</v>
+      </c>
+      <c r="T7" s="6">
+        <f t="shared" ref="T7:T13" si="5">L7</f>
+        <v>53.9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -11007,8 +11147,40 @@
         <f t="shared" si="0"/>
         <v>86.571035064133454</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J8" t="s">
+        <v>3</v>
+      </c>
+      <c r="K8">
+        <v>25.8</v>
+      </c>
+      <c r="L8">
+        <v>49.6</v>
+      </c>
+      <c r="M8">
+        <v>6.3</v>
+      </c>
+      <c r="N8">
+        <v>41.5</v>
+      </c>
+      <c r="P8" s="19">
+        <f t="shared" si="2"/>
+        <v>56.497999818602068</v>
+      </c>
+      <c r="Q8" s="6">
+        <f t="shared" si="3"/>
+        <v>25.8</v>
+      </c>
+      <c r="R8" s="6"/>
+      <c r="S8" s="19">
+        <f t="shared" si="4"/>
+        <v>86.571035064133454</v>
+      </c>
+      <c r="T8" s="6">
+        <f t="shared" si="5"/>
+        <v>49.6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -11036,8 +11208,40 @@
         <f t="shared" si="0"/>
         <v>92.347382263528885</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J9" t="s">
+        <v>20</v>
+      </c>
+      <c r="K9">
+        <v>37.6</v>
+      </c>
+      <c r="L9">
+        <v>60.7</v>
+      </c>
+      <c r="M9">
+        <v>17.8</v>
+      </c>
+      <c r="N9">
+        <v>51.6</v>
+      </c>
+      <c r="P9" s="19">
+        <f t="shared" si="2"/>
+        <v>57.246566631171873</v>
+      </c>
+      <c r="Q9" s="6">
+        <f t="shared" si="3"/>
+        <v>37.6</v>
+      </c>
+      <c r="R9" s="6"/>
+      <c r="S9" s="19">
+        <f t="shared" si="4"/>
+        <v>92.347382263528885</v>
+      </c>
+      <c r="T9" s="6">
+        <f t="shared" si="5"/>
+        <v>60.7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>21</v>
       </c>
@@ -11065,8 +11269,40 @@
         <f t="shared" si="0"/>
         <v>107.93979016539292</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J10" t="s">
+        <v>21</v>
+      </c>
+      <c r="K10">
+        <v>58.9</v>
+      </c>
+      <c r="L10">
+        <v>85.5</v>
+      </c>
+      <c r="M10">
+        <v>48.8</v>
+      </c>
+      <c r="N10">
+        <v>78.3</v>
+      </c>
+      <c r="P10" s="19">
+        <f t="shared" si="2"/>
+        <v>59.783034890110805</v>
+      </c>
+      <c r="Q10" s="6">
+        <f t="shared" si="3"/>
+        <v>58.9</v>
+      </c>
+      <c r="R10" s="6"/>
+      <c r="S10" s="19">
+        <f t="shared" si="4"/>
+        <v>107.93979016539292</v>
+      </c>
+      <c r="T10" s="6">
+        <f t="shared" si="5"/>
+        <v>85.5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>22</v>
       </c>
@@ -11094,8 +11330,40 @@
         <f t="shared" si="0"/>
         <v>107.51085018565145</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J11" t="s">
+        <v>22</v>
+      </c>
+      <c r="K11">
+        <v>71.599999999999994</v>
+      </c>
+      <c r="L11">
+        <v>104.8</v>
+      </c>
+      <c r="M11">
+        <v>56.8</v>
+      </c>
+      <c r="N11">
+        <v>81.900000000000006</v>
+      </c>
+      <c r="P11" s="19">
+        <f t="shared" si="2"/>
+        <v>67.291815900739664</v>
+      </c>
+      <c r="Q11" s="6">
+        <f t="shared" si="3"/>
+        <v>71.599999999999994</v>
+      </c>
+      <c r="R11" s="6"/>
+      <c r="S11" s="19">
+        <f t="shared" si="4"/>
+        <v>107.51085018565145</v>
+      </c>
+      <c r="T11" s="6">
+        <f t="shared" si="5"/>
+        <v>104.8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -11123,8 +11391,40 @@
         <f t="shared" si="0"/>
         <v>98.941412614337224</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="J12" t="s">
+        <v>13</v>
+      </c>
+      <c r="K12">
+        <v>53.5</v>
+      </c>
+      <c r="L12">
+        <v>89.7</v>
+      </c>
+      <c r="M12">
+        <v>41</v>
+      </c>
+      <c r="N12">
+        <v>69</v>
+      </c>
+      <c r="P12" s="19">
+        <f t="shared" si="2"/>
+        <v>68.661257418652681</v>
+      </c>
+      <c r="Q12" s="6">
+        <f t="shared" si="3"/>
+        <v>53.5</v>
+      </c>
+      <c r="R12" s="6"/>
+      <c r="S12" s="19">
+        <f t="shared" si="4"/>
+        <v>98.941412614337224</v>
+      </c>
+      <c r="T12" s="6">
+        <f t="shared" si="5"/>
+        <v>89.7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>14</v>
       </c>
@@ -11151,6 +11451,38 @@
       <c r="H13" s="17">
         <f t="shared" si="0"/>
         <v>94.953451257263765</v>
+      </c>
+      <c r="J13" t="s">
+        <v>14</v>
+      </c>
+      <c r="K13">
+        <v>53.9</v>
+      </c>
+      <c r="L13">
+        <v>73.3</v>
+      </c>
+      <c r="M13">
+        <v>39.4</v>
+      </c>
+      <c r="N13">
+        <v>64.3</v>
+      </c>
+      <c r="P13" s="19">
+        <f t="shared" si="2"/>
+        <v>65.982148506817737</v>
+      </c>
+      <c r="Q13" s="6">
+        <f t="shared" si="3"/>
+        <v>53.9</v>
+      </c>
+      <c r="R13" s="6"/>
+      <c r="S13" s="19">
+        <f t="shared" si="4"/>
+        <v>94.953451257263765</v>
+      </c>
+      <c r="T13" s="6">
+        <f t="shared" si="5"/>
+        <v>73.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update energy rates to discuss differences between the Yackulic and Rind price data sets
</commit_message>
<xml_diff>
--- a/Energy Rates_2014.xlsx
+++ b/Energy Rates_2014.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15A8B50D-F342-432E-85B9-4CCBC0B3A35E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEBC657E-833C-4249-B8B4-4A1EEDB48EC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-1260" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="12" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="43">
   <si>
     <t>Price Profiles for Generation Shaping ($/MWh)--Simulation Info Tab, Monday Hourly Values</t>
   </si>
@@ -164,6 +164,12 @@
   <si>
     <t>On-peak</t>
   </si>
+  <si>
+    <t>Off-peak</t>
+  </si>
+  <si>
+    <t>Rind - Yackulic</t>
+  </si>
 </sst>
 </file>
 
@@ -277,10 +283,10 @@
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -10909,7 +10915,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E4AFA8A-3ECC-44AF-AF5D-50FFF5439E6C}">
-  <dimension ref="A1:T13"/>
+  <dimension ref="A1:W13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="7" max="7" width="8.81640625" bestFit="1" customWidth="1"/>
@@ -10917,17 +10923,17 @@
     <col min="18" max="18" width="2.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>24</v>
       </c>
@@ -10946,8 +10952,11 @@
       <c r="S4" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="5" spans="1:20" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="V4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
         <v>16</v>
       </c>
@@ -10996,8 +11005,14 @@
       <c r="T5" s="8" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="V5" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="W5" s="8" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -11040,7 +11055,7 @@
       <c r="N6">
         <v>46.2</v>
       </c>
-      <c r="P6" s="19">
+      <c r="P6" s="18">
         <f>G6</f>
         <v>64.699513831553674</v>
       </c>
@@ -11049,7 +11064,7 @@
         <v>39.5</v>
       </c>
       <c r="R6" s="6"/>
-      <c r="S6" s="19">
+      <c r="S6" s="18">
         <f>H6</f>
         <v>88.52242346956902</v>
       </c>
@@ -11057,8 +11072,16 @@
         <f>L6</f>
         <v>53.3</v>
       </c>
-    </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="V6" s="4">
+        <f>P6-Q6</f>
+        <v>25.199513831553674</v>
+      </c>
+      <c r="W6" s="4">
+        <f>S6-T6</f>
+        <v>35.222423469569023</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -11101,7 +11124,7 @@
       <c r="N7">
         <v>46.3</v>
       </c>
-      <c r="P7" s="19">
+      <c r="P7" s="18">
         <f t="shared" ref="P7:P13" si="2">G7</f>
         <v>60.742340534310571</v>
       </c>
@@ -11110,7 +11133,7 @@
         <v>33.5</v>
       </c>
       <c r="R7" s="6"/>
-      <c r="S7" s="19">
+      <c r="S7" s="18">
         <f t="shared" ref="S7:S13" si="4">H7</f>
         <v>85.050518027815997</v>
       </c>
@@ -11118,8 +11141,16 @@
         <f t="shared" ref="T7:T13" si="5">L7</f>
         <v>53.9</v>
       </c>
-    </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="V7" s="4">
+        <f t="shared" ref="V7:V13" si="6">P7-Q7</f>
+        <v>27.242340534310571</v>
+      </c>
+      <c r="W7" s="4">
+        <f t="shared" ref="W7:W13" si="7">S7-T7</f>
+        <v>31.150518027815998</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -11162,7 +11193,7 @@
       <c r="N8">
         <v>41.5</v>
       </c>
-      <c r="P8" s="19">
+      <c r="P8" s="18">
         <f t="shared" si="2"/>
         <v>56.497999818602068</v>
       </c>
@@ -11171,7 +11202,7 @@
         <v>25.8</v>
       </c>
       <c r="R8" s="6"/>
-      <c r="S8" s="19">
+      <c r="S8" s="18">
         <f t="shared" si="4"/>
         <v>86.571035064133454</v>
       </c>
@@ -11179,8 +11210,16 @@
         <f t="shared" si="5"/>
         <v>49.6</v>
       </c>
-    </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="V8" s="4">
+        <f t="shared" si="6"/>
+        <v>30.697999818602067</v>
+      </c>
+      <c r="W8" s="4">
+        <f t="shared" si="7"/>
+        <v>36.971035064133453</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -11223,7 +11262,7 @@
       <c r="N9">
         <v>51.6</v>
       </c>
-      <c r="P9" s="19">
+      <c r="P9" s="18">
         <f t="shared" si="2"/>
         <v>57.246566631171873</v>
       </c>
@@ -11232,7 +11271,7 @@
         <v>37.6</v>
       </c>
       <c r="R9" s="6"/>
-      <c r="S9" s="19">
+      <c r="S9" s="18">
         <f t="shared" si="4"/>
         <v>92.347382263528885</v>
       </c>
@@ -11240,8 +11279,16 @@
         <f t="shared" si="5"/>
         <v>60.7</v>
       </c>
-    </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="V9" s="4">
+        <f t="shared" si="6"/>
+        <v>19.646566631171872</v>
+      </c>
+      <c r="W9" s="4">
+        <f t="shared" si="7"/>
+        <v>31.647382263528883</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>21</v>
       </c>
@@ -11284,7 +11331,7 @@
       <c r="N10">
         <v>78.3</v>
       </c>
-      <c r="P10" s="19">
+      <c r="P10" s="18">
         <f t="shared" si="2"/>
         <v>59.783034890110805</v>
       </c>
@@ -11293,7 +11340,7 @@
         <v>58.9</v>
       </c>
       <c r="R10" s="6"/>
-      <c r="S10" s="19">
+      <c r="S10" s="18">
         <f t="shared" si="4"/>
         <v>107.93979016539292</v>
       </c>
@@ -11301,8 +11348,16 @@
         <f t="shared" si="5"/>
         <v>85.5</v>
       </c>
-    </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="V10" s="4">
+        <f t="shared" si="6"/>
+        <v>0.88303489011080671</v>
+      </c>
+      <c r="W10" s="4">
+        <f t="shared" si="7"/>
+        <v>22.439790165392921</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>22</v>
       </c>
@@ -11345,7 +11400,7 @@
       <c r="N11">
         <v>81.900000000000006</v>
       </c>
-      <c r="P11" s="19">
+      <c r="P11" s="18">
         <f t="shared" si="2"/>
         <v>67.291815900739664</v>
       </c>
@@ -11354,7 +11409,7 @@
         <v>71.599999999999994</v>
       </c>
       <c r="R11" s="6"/>
-      <c r="S11" s="19">
+      <c r="S11" s="18">
         <f t="shared" si="4"/>
         <v>107.51085018565145</v>
       </c>
@@ -11362,8 +11417,16 @@
         <f t="shared" si="5"/>
         <v>104.8</v>
       </c>
-    </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="V11" s="4">
+        <f t="shared" si="6"/>
+        <v>-4.3081840992603304</v>
+      </c>
+      <c r="W11" s="4">
+        <f t="shared" si="7"/>
+        <v>2.7108501856514522</v>
+      </c>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -11406,7 +11469,7 @@
       <c r="N12">
         <v>69</v>
       </c>
-      <c r="P12" s="19">
+      <c r="P12" s="18">
         <f t="shared" si="2"/>
         <v>68.661257418652681</v>
       </c>
@@ -11415,7 +11478,7 @@
         <v>53.5</v>
       </c>
       <c r="R12" s="6"/>
-      <c r="S12" s="19">
+      <c r="S12" s="18">
         <f t="shared" si="4"/>
         <v>98.941412614337224</v>
       </c>
@@ -11423,8 +11486,16 @@
         <f t="shared" si="5"/>
         <v>89.7</v>
       </c>
-    </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="V12" s="4">
+        <f t="shared" si="6"/>
+        <v>15.161257418652681</v>
+      </c>
+      <c r="W12" s="4">
+        <f t="shared" si="7"/>
+        <v>9.2414126143372215</v>
+      </c>
+    </row>
+    <row r="13" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>14</v>
       </c>
@@ -11467,7 +11538,7 @@
       <c r="N13">
         <v>64.3</v>
       </c>
-      <c r="P13" s="19">
+      <c r="P13" s="18">
         <f t="shared" si="2"/>
         <v>65.982148506817737</v>
       </c>
@@ -11476,13 +11547,21 @@
         <v>53.9</v>
       </c>
       <c r="R13" s="6"/>
-      <c r="S13" s="19">
+      <c r="S13" s="18">
         <f t="shared" si="4"/>
         <v>94.953451257263765</v>
       </c>
       <c r="T13" s="6">
         <f t="shared" si="5"/>
         <v>73.3</v>
+      </c>
+      <c r="V13" s="4">
+        <f t="shared" si="6"/>
+        <v>12.082148506817738</v>
+      </c>
+      <c r="W13" s="4">
+        <f t="shared" si="7"/>
+        <v>21.653451257263768</v>
       </c>
     </row>
   </sheetData>
@@ -14029,19 +14108,19 @@
       <c r="E4" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="18" t="s">
+      <c r="F4" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="G4" s="18"/>
-      <c r="H4" s="18"/>
+      <c r="G4" s="19"/>
+      <c r="H4" s="19"/>
       <c r="I4" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="J4" s="18" t="s">
+      <c r="J4" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="K4" s="18"/>
-      <c r="L4" s="18"/>
+      <c r="K4" s="19"/>
+      <c r="L4" s="19"/>
       <c r="M4" s="6"/>
     </row>
     <row r="5" spans="2:13" x14ac:dyDescent="0.35">

</xml_diff>